<commit_message>
Update Personal Tool Journey: refresh racing line chart, data, and add presentation plots export
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Personal Tool Journey/ronsAnalyticsToolsOverTime.xlsx
+++ b/Personal Tool Journey/ronsAnalyticsToolsOverTime.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rnguymon/Library/CloudStorage/Box-Box/AAA Intensive Data Analytic Workshop/DATA_2026/Data Storytelling/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rnguymon/Library/CloudStorage/Box-Box/RonsPortfolio/Personal Tool Journey/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF5EF019-7AF7-7349-8AA8-6807B063FB06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F01E60-0F4C-2047-B9B3-183213C43BF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-30220" yWindow="1900" windowWidth="28040" windowHeight="17440" xr2:uid="{38818B61-A50B-4C4A-A1B6-5C4444C9EB93}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
   <si>
     <t>Minitab</t>
   </si>
@@ -78,9 +78,6 @@
   </si>
   <si>
     <t>Authoring with McGraw-Hill</t>
-  </si>
-  <si>
-    <t>McGraw-Hill Business Analytics and Statistics Innovation Summit</t>
   </si>
   <si>
     <t>Working on Bachelors degree</t>
@@ -146,9 +143,6 @@
     <t>More authoring</t>
   </si>
   <si>
-    <t>MH Summit</t>
-  </si>
-  <si>
     <t>ShortEvent</t>
   </si>
   <si>
@@ -159,6 +153,18 @@
   </si>
   <si>
     <t>DATA</t>
+  </si>
+  <si>
+    <t>McGraw-Hill Business Analytics and Statistics Innovation Summit Tampa</t>
+  </si>
+  <si>
+    <t>MH Summit Tampa</t>
+  </si>
+  <si>
+    <t>McGraw-Hill Business Analytics and Statistics Innovation Summit Nashville</t>
+  </si>
+  <si>
+    <t>MH Summit Nashville</t>
   </si>
 </sst>
 </file>
@@ -532,7 +538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01C9F51E-103C-384A-BA63-A88EB993FEA9}">
-  <dimension ref="A1:O341"/>
+  <dimension ref="A1:O343"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
@@ -543,7 +549,7 @@
         <v>12</v>
       </c>
       <c r="C1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D1" t="s">
         <v>3</v>
@@ -579,7 +585,7 @@
         <v>11</v>
       </c>
       <c r="O1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
@@ -587,10 +593,10 @@
         <v>35916</v>
       </c>
       <c r="B2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
@@ -732,10 +738,10 @@
         <v>36404</v>
       </c>
       <c r="B18" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C18" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D18">
         <v>10</v>
@@ -1023,10 +1029,10 @@
         <v>37073</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D40">
         <v>18</v>
@@ -1184,10 +1190,10 @@
         <v>37469</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C53" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D53">
         <v>31</v>
@@ -1669,10 +1675,10 @@
         <v>38687</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C93" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D93">
         <v>71</v>
@@ -2148,10 +2154,10 @@
         <v>39692</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C126" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D126">
         <v>89</v>
@@ -3200,10 +3206,10 @@
         <v>42186</v>
       </c>
       <c r="B208" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C208" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D208">
         <v>171</v>
@@ -3628,10 +3634,10 @@
         <v>43040</v>
       </c>
       <c r="B236" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C236" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D236">
         <v>130</v>
@@ -3801,10 +3807,10 @@
         <v>43344</v>
       </c>
       <c r="B246" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C246" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D246">
         <v>110</v>
@@ -3890,7 +3896,7 @@
         <v>43466</v>
       </c>
       <c r="B250" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D250">
         <v>102</v>
@@ -4975,7 +4981,7 @@
         <v>13</v>
       </c>
       <c r="C294" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D294">
         <v>230</v>
@@ -5337,7 +5343,7 @@
         <v>45170</v>
       </c>
       <c r="B306" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D306">
         <v>230</v>
@@ -5819,10 +5825,10 @@
         <v>45658</v>
       </c>
       <c r="B322" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C322" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D322">
         <v>230</v>
@@ -6181,10 +6187,10 @@
         <v>46023</v>
       </c>
       <c r="B334" s="1" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
       <c r="C334" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D334">
         <v>230</v>
@@ -6378,10 +6384,10 @@
         <v>46235</v>
       </c>
       <c r="B341" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C341" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D341">
         <v>200</v>
@@ -6403,6 +6409,64 @@
       </c>
       <c r="O341">
         <v>800</v>
+      </c>
+    </row>
+    <row r="342" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A342" s="1">
+        <v>46266</v>
+      </c>
+      <c r="D342">
+        <v>200</v>
+      </c>
+      <c r="F342">
+        <v>50</v>
+      </c>
+      <c r="I342">
+        <v>1300</v>
+      </c>
+      <c r="K342">
+        <v>160</v>
+      </c>
+      <c r="M342">
+        <v>1500</v>
+      </c>
+      <c r="N342">
+        <v>360</v>
+      </c>
+      <c r="O342">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="343" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A343" s="1">
+        <v>46296</v>
+      </c>
+      <c r="B343" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C343" t="s">
+        <v>42</v>
+      </c>
+      <c r="D343">
+        <v>200</v>
+      </c>
+      <c r="F343">
+        <v>50</v>
+      </c>
+      <c r="I343">
+        <v>1400</v>
+      </c>
+      <c r="K343">
+        <v>170</v>
+      </c>
+      <c r="M343">
+        <v>1500</v>
+      </c>
+      <c r="N343">
+        <v>360</v>
+      </c>
+      <c r="O343">
+        <v>1200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>